<commit_message>
PLAN_PROJ_V2 Phase 77: Projektsteckbrief mit Ableitung aus Erfassung und Auftrag
- Blatt Steckbrief in projektierung_logik_v1.xlsx (34 Startregeln; Syntax:
  fester Text, leer = Antwort 1:1, Mapping Antwort->Text | *->Text)
- SteckbriefWert-Tabelle + steckbrief_ableiten/steckbrief_daten im Kern
  (erste passende Regel je Feld, manuell geaenderte Felder geschuetzt,
  fp_frage fuer Phase 80 vorbereitet)
- Ableitung bei Projektanlage + Knopf Neu ableiten; Felder per Klick
  editierbar (manuell-Kennzeichen)
- Steckbrief-Block oben in der Projektakte und in der Vorgangsakte nach
  Auftrag (Vertrieb read-only); pj-steck-Styles zuerst im Prototyp
- Phasentest 43/43, Unit-Suite 117/117

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projektierung_logik_v1.xlsx
+++ b/projektierung_logik_v1.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Paketregeln" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Ordnerstruktur" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Sub-Typen" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Steckbrief" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -511,7 +512,6 @@
           <t>Auftragsunterlagen prüfen (Angebot, Protokoll, Fotos)</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -552,7 +552,6 @@
           <t>Kunde kontaktieren, Ablauf erklären, Feinplanungstermin abstimmen</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -593,7 +592,6 @@
           <t>Auftrag in TAIFUN anlegen</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>innendienst</t>
@@ -634,7 +632,6 @@
           <t>Anzahlungsrechnung veranlassen</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>buchhaltung</t>
@@ -675,7 +672,6 @@
           <t>Feinplanungstermin vor Ort durchführen</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>feinplaner</t>
@@ -716,7 +712,6 @@
           <t>Heizlast berechnen (Heizreport) und Ergebnis eintragen</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>feinplaner</t>
@@ -757,7 +752,6 @@
           <t>Fotos Außengerät/Heizungsraum/Zählerschrank abgelegt</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>feinplaner</t>
@@ -798,7 +792,6 @@
           <t>Abweichungen zum Angebot prüfen, ggf. Nachtrag (Überarbeiten)</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -839,7 +832,6 @@
           <t>Gerät/Paket final festgelegt</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -880,7 +872,6 @@
           <t>Zählerschrank/Unterverteilung bewerten</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>elektroplaner</t>
@@ -921,7 +912,6 @@
           <t>Leitungsweg und Querschnitt festlegen</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
           <t>elektroplaner</t>
@@ -962,7 +952,6 @@
           <t>Netzbetreiber-Anmeldung WP (§14a) einreichen</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>elektroplaner</t>
@@ -1006,7 +995,6 @@
           <t>Zustimmung Netzbetreiber liegt vor</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>elektroplaner</t>
@@ -1047,7 +1035,6 @@
           <t>Elektro-Team einplanen oder externen Elektriker beauftragen</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>elektroplaner</t>
@@ -1088,7 +1075,6 @@
           <t>Stückliste prüfen</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -1129,7 +1115,6 @@
           <t>Material bei Collin bestellen</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -1170,7 +1155,6 @@
           <t>Liefertermin bestätigt</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -1211,7 +1195,6 @@
           <t>Wareneingang geprüft</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -1252,7 +1235,6 @@
           <t>Kunde Tarifvertrag SpotDynamic unterschreiben lassen</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -1293,7 +1275,6 @@
           <t>Smart-Meter-/iMSys-Bestellung beim Partner auslösen</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -1334,7 +1315,6 @@
           <t>Zählerwechsel-Termin mit Netzbetreiber/Partner</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -1378,7 +1358,6 @@
           <t>iMSys eingebaut, Zählernummer eingetragen</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
           <t>montage</t>
@@ -1419,7 +1398,6 @@
           <t>HEMS eingerichtet und mit WP verbunden</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
           <t>montage</t>
@@ -1460,7 +1438,6 @@
           <t>Tarifstart bestätigt</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -1504,7 +1481,6 @@
           <t>Kunde in App eingewiesen</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
           <t>montage</t>
@@ -1545,7 +1521,6 @@
           <t>Fundamentmaße aus Gerätedaten festlegen</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -1586,7 +1561,6 @@
           <t>GaLa-Bau beauftragen (Mail mit Fotos)</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -1627,7 +1601,6 @@
           <t>Fundamenttermin bestätigt</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -1668,7 +1641,6 @@
           <t>Fundament fertig, Foto abgelegt</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -1709,7 +1681,6 @@
           <t>Entsorger beauftragen (Mail mit Fotos, Tankgröße, Zugang)</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -1750,7 +1721,6 @@
           <t>Termin vor Montage bestätigt</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -1791,7 +1761,6 @@
           <t>Entsorgungsnachweis abgelegt</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -1832,7 +1801,6 @@
           <t>Lift/Kran bestellen</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -1873,7 +1841,6 @@
           <t>Stellfläche/Straßensperrung geklärt</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -1914,7 +1881,6 @@
           <t>Statik/Tragfähigkeit prüfen</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -1955,7 +1921,6 @@
           <t>Dachdecker beauftragen</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -1996,7 +1961,6 @@
           <t>BzA (Bestätigung zum Antrag) an Kunden</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
           <t>innendienst</t>
@@ -2037,7 +2001,6 @@
           <t>Förderantrag durch Kunden gestellt (Nachweis)</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -2081,7 +2044,6 @@
           <t>Zusage liegt vor</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -2122,7 +2084,6 @@
           <t>BnD nach Abnahme erstellt</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
           <t>innendienst</t>
@@ -2163,7 +2124,6 @@
           <t>Montagetermin mit Kunde vereinbart und bestätigt</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -2204,7 +2164,6 @@
           <t>Teams zugewiesen</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -2245,7 +2204,6 @@
           <t>Steckbrief für Montage geprüft</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -2286,7 +2244,6 @@
           <t>Montagebericht liegt vor</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
           <t>montage</t>
@@ -2327,7 +2284,6 @@
           <t>Inbetriebnahmeprotokoll liegt vor</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
           <t>montage</t>
@@ -2368,7 +2324,6 @@
           <t>Abnahmeprotokoll mit Kundenunterschrift</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
           <t>montage</t>
@@ -2409,7 +2364,6 @@
           <t>Restarbeiten/Reklamationen erfasst</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -2450,7 +2404,6 @@
           <t>Rechnung freigegeben</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -2491,7 +2444,6 @@
           <t>Feinplanung Dach/Strang/Speicherort</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
           <t>feinplaner</t>
@@ -2532,7 +2484,6 @@
           <t>Netzanschlussbegehren beim Netzbetreiber</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
           <t>elektroplaner</t>
@@ -2576,7 +2527,6 @@
           <t>Gerüst bestellen</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -2617,7 +2567,6 @@
           <t>Material bestellen</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -2658,7 +2607,6 @@
           <t>Inbetriebnahme + Fertigmeldung Netzbetreiber</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
           <t>elektroplaner</t>
@@ -2699,7 +2647,6 @@
           <t>Marktstammdatenregister eingetragen</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
           <t>elektroplaner</t>
@@ -2740,7 +2687,6 @@
           <t>Wallbox beim Netzbetreiber anmelden</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
           <t>elektroplaner</t>
@@ -2781,7 +2727,6 @@
           <t>Material bestellen</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -2822,7 +2767,6 @@
           <t>Montage + Protokoll</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
           <t>montage</t>
@@ -2863,7 +2807,6 @@
           <t>Feinplanung Innen-/Außengerät, Leitungsweg, Kondensat</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
           <t>feinplaner</t>
@@ -2904,7 +2847,6 @@
           <t>Material bestellen</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
           <t>projektierer</t>
@@ -2945,7 +2887,6 @@
           <t>Montage + Inbetriebnahme (Kältemittel-Nachweis)</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
           <t>montage</t>
@@ -3556,4 +3497,935 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>feld</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>sparte</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>quelle_typ</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>quelle</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>wert_oder_regel</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>hersteller</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>030/031/045-056</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Bosch</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>leistungsklasse</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>030/031</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>15 kW (Serie CS8800i)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>leistungsklasse</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>045/050</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>4 kW (CS3800i)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>leistungsklasse</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>046/051</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>6 kW (CS3800i)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>leistungsklasse</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>047/052</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>7 kW (CS3800i)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>leistungsklasse</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>048/053</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>10 kW (CS3800i)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>leistungsklasse</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>049/054</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>13 kW (CS3800i)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>innengeraet</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>055</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>AWMB (integrierter 70-l-Puffer)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>innengeraet</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>056</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>AWE + externer Puffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>innengeraet</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>045-049</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>AWM (Warmwasserspeicher 180 l integriert)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>innengeraet</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>050-054</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>AWE</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>warmwasser</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>069</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>390-l-Solarspeicher (bivalent, Solarthermie-Uebernahme)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>warmwasser</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>065</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>300-l-Warmwasserspeicher</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>warmwasser</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>frage</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>N02</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Nein→ohne Warmwasser | Ja→ueber die Waermepumpe</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>aufstellort</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>010</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Boden (Fundament wird erstellt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>aufstellort</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>132</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Garagendach (Bodenkonsole)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>aufstellort</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>frage</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>N04</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>zaehlerschrank</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>frage</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>E03</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2-Feld→wird erneuert: Zweifeld | 3-Feld→wird erneuert: Dreifeld | 4-Feld und mehr→wird erneuert: Vierfeld</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>zaehlerschrank</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>152</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>bleibt · Unterverteilung wird gesetzt</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>zaehlerschrank</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>frage</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>E02</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Nein→bleibt</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>oeltank</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>frage</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>A07</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Nein→nein | Ja→ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>oeltank_groesse</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>frage</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>A09</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>oeltank_groesse</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>frage</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>A19</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>oeltank_material</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>frage</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>A08</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>alte_anlage</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>frage</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>A01</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>alte_anlage_standort</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>frage</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>A04</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>DG→Dachzentrale (DG) | *→</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>hems</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>frage</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Ja→ja | Nein→nein</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>imsys</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>frage</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Ja→ja | Nein→nein</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>dyn_tarif</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>frage</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>P03</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Ja→ja | Nein→nein</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>kran</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>frage</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>N09</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Ja→Mobiler Kran eingeplant | Nein→nicht erforderlich</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>kran</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>135</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Kran als Eventualposition im Angebot</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>besonderheiten</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Z24</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Solarthermie wird stillgelegt (Z24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>besonderheiten</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>frage</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>A12</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>dach</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>frage</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>PV01</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
PLAN_PROJ_V2 Phase 82: Montage-Backend mit Formularen, Galerie und Wochenkalender
- Startseite /montage: Team-Auswahl, chronologische Liste (Heute/Woche/
  Danach, Vergangenes eingeklappt) und mobiler Wochenkalender je Team
- Auftragsdetail: Steckbrief read-only, Ansprechpartner Friondo, Teams/
  Subs mit Terminen, komplette Vorgangs-Galerie (8 Ordner, ansehen +
  aufnehmen), Restarbeiten melden (Text + Foto), keine Preise
- Galerie-Rechte: Rolle montage erreicht nur Datei-/Upload-Route, geprueft
  gegen die eigenen Team-Einsaetze; loeschen/verschieben gesperrt
- Blatt Formulare (Montagebericht, Inbetriebnahme-, Abnahmeprotokoll, 49
  Felder) + generische mobile Formular-Runtime mit Zwischenspeichern,
  Foto-Feldern (in Galerie) und Canvas-Unterschrift; Abschluss = PDF in
  Galerie Inbetrieb-/Abnahme + Aufgabe erledigt + Restarbeiten aus
  Maengel-Zeilen des Abnahmeprotokolls
- Phasentest 28/28, Unit-Suite 117/117

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projektierung_logik_v1.xlsx
+++ b/projektierung_logik_v1.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Fragen FP-WP" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Steckbrief" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Stücklisten" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Formulare" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3564,13 +3565,11 @@
           <t>ja_nein</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3593,13 +3592,11 @@
           <t>zahl</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3622,7 +3619,6 @@
           <t>text</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>J</t>
@@ -3655,7 +3651,6 @@
           <t>ja_nein</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>J</t>
@@ -3688,13 +3683,11 @@
           <t>text</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3754,13 +3747,11 @@
           <t>ja_nein</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3783,7 +3774,6 @@
           <t>ja_nein</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>J</t>
@@ -3816,13 +3806,11 @@
           <t>ja_nein</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3845,7 +3833,6 @@
           <t>ja_nein</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>J</t>
@@ -3878,7 +3865,6 @@
           <t>text</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>N</t>
@@ -3911,7 +3897,6 @@
           <t>text</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>N</t>
@@ -3944,13 +3929,11 @@
           <t>text</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3973,13 +3956,11 @@
           <t>ja_nein</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4002,13 +3983,11 @@
           <t>zahl</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4041,7 +4020,6 @@
           <t>J</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4105,7 +4083,6 @@
           <t>FP-A01</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4209,7 +4186,6 @@
           <t>FP-O02</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4232,7 +4208,6 @@
           <t>FP-O03</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4309,7 +4284,6 @@
           <t>FP-H01</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5363,4 +5337,1684 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G50"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>formular</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>seite</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>feld_key</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>bezeichnung</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>typ</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>pflicht</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>optionen</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>montagebericht</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Einsatz</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>mb_datum</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Datum</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>datum</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>montagebericht</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Einsatz</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>mb_mitarbeiter</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Mitarbeiter (Team)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>montagebericht</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Einsatz</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>mb_beginn</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Arbeitsbeginn (Uhrzeit)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>montagebericht</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Einsatz</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>mb_ende</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Arbeitsende (Uhrzeit)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>montagebericht</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Ausgeführte Arbeiten</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>mb_altanlage</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Altanlage demontiert</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>montagebericht</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ausgeführte Arbeiten</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>mb_aussengeraet</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Außengerät gesetzt</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>montagebericht</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Ausgeführte Arbeiten</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>mb_innengeraet</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Innengerät montiert</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>montagebericht</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Ausgeführte Arbeiten</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>mb_hydraulik</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Hydraulik angeschlossen</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>montagebericht</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Ausgeführte Arbeiten</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>mb_elektro</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Elektro angeschlossen</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>montagebericht</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Ausgeführte Arbeiten</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>mb_zaehlerschrank</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Zählerschrank</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>montagebericht</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Ausgeführte Arbeiten</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>mb_puffer_ww</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Puffer / Warmwasser</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>montagebericht</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Ausgeführte Arbeiten</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>mb_kondensat</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Kondensat</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>montagebericht</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Ausgeführte Arbeiten</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>mb_daemmung</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Dämmung</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>montagebericht</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Ausgeführte Arbeiten</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>mb_folierung</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Folierung</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>montagebericht</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Abweichungen &amp; Material</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>mb_abweichungen</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Abweichungen / Mehrleistungen</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>montagebericht</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Abweichungen &amp; Material</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>mb_abweichung_foto</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Foto zur Abweichung</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>foto</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Inbetrieb-/Abnahme</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>montagebericht</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Abweichungen &amp; Material</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>mb_nachbestellung</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Materialnachbestellung</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>montagebericht</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Abweichungen &amp; Material</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>mb_regie</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Stunden Regie</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>zahl</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>montagebericht</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Abweichungen &amp; Material</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>mb_foto_anlage</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Foto Neue Anlage</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>foto</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Neue Anlage</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>inbetriebnahme</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Gerät</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>ib_sn_aussen</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Seriennummer Außengerät</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>inbetriebnahme</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Gerät</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>ib_sn_innen</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Seriennummer Innengerät</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>inbetriebnahme</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Gerät</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ib_sn_puffer</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Seriennummer Puffer/Speicher</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>inbetriebnahme</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Gerät</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ib_kaeltemittel</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Kältemittel / Füllmenge</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>inbetriebnahme</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Gerät</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>ib_dichtheit</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Dichtheitsprüfung bestanden</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>inbetriebnahme</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Hydraulik</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>ib_spuelung</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Spülung/Befüllung durchgeführt</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>inbetriebnahme</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Hydraulik</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ib_druck</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Anlagendruck (bar)</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>zahl</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>inbetriebnahme</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Hydraulik</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>ib_vorlauf</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Vorlauftemperatur (°C)</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>zahl</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>inbetriebnahme</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Hydraulik</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>ib_heizkurve</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Heizkurve</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>inbetriebnahme</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Hydraulik</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>ib_abgleich</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Hydraulischer Abgleich durchgeführt</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>inbetriebnahme</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Hydraulik</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>ib_frostschutz</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Frostschutz</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>inbetriebnahme</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Elektrik</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ib_rcd</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>RCD-Prüfung bestanden</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>inbetriebnahme</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Elektrik</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>ib_iso</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Isolationswiderstand</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>inbetriebnahme</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Elektrik</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ib_schleife</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Schleifenimpedanz</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>inbetriebnahme</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Elektrik</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>ib_zaehlernummer</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Zählernummer / iMSys</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>inbetriebnahme</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Elektrik</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>ib_hems</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>HEMS verbunden</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>inbetriebnahme</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Abschluss</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ib_probelauf</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Probelauf ok</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>inbetriebnahme</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Abschluss</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>ib_einweisung</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Einweisung Kunde</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>inbetriebnahme</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Abschluss</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>ib_einweisung_dauer</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Dauer der Einweisung (Minuten)</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>zahl</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>inbetriebnahme</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Abschluss</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>ib_bemerkung</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Bemerkungen</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>inbetriebnahme</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Abschluss</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ib_unterschrift_monteur</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Unterschrift Monteur</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>unterschrift</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>abnahme</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Leistung</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>ab_vollstaendig</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Leistungen vollständig erbracht</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>abnahme</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Leistung</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>ab_maengel</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Mängel / Restarbeiten (eine je Zeile – wird als Restarbeiten-Liste übernommen)</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>abnahme</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Leistung</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>ab_maengel_foto</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Foto zu Mängeln</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>foto</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Inbetrieb-/Abnahme</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>abnahme</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Leistung</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>ab_frist</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Frist für Restarbeiten</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>datum</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>abnahme</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Übergabe</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>ab_unterlagen</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Unterlagen übergeben (Bedienungsanleitung, Garantie, Protokolle)</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>abnahme</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Übergabe</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>ab_einweisung_bestaetigt</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Kunde bestätigt Einweisung</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>abnahme</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Unterschriften</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>ab_datum</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Datum</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>datum</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>abnahme</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Unterschriften</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>ab_unterschrift_kunde</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Unterschrift Kunde</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>unterschrift</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>abnahme</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Unterschriften</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>ab_unterschrift_monteur</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Unterschrift Monteur</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>unterschrift</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Paket Foerderung entfaellt; BnD-Punkt wandert nach Abnahme & Freigabe
Andreas 27.09.2026: Oberbegriff Foerderung in der Projektakte komplett
raus; BnD nach Abnahme erstellt als Schritt 6 (M+10) im Paket
Abnahme & Freigabe.

- Blatt Aufgabenpakete + Paketregeln angepasst (Validierung gruen),
  Foerderung aus der Paket-Rangfolge entfernt
- Migration migration_bnd_abnahme: Foerderungs-Instanzen samt Aufgaben
  geloescht (28 lokal), BnD-Punkt an aktive Abnahme-Instanzen gehaengt
  (5 lokal, erledigter Status wuerde uebernommen); idempotent, doppelt
  gelaufen
- Neuanlage geprueft: 7 Pakete ohne Foerderung, Abnahme & Freigabe mit
  6 Schritten inkl. BnD; Unit-Suite 117/117

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projektierung_logik_v1.xlsx
+++ b/projektierung_logik_v1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P48"/>
+  <dimension ref="A1:P46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1700,17 +1700,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>foerderung</t>
+          <t>montagevorbereitung</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Förderung</t>
+          <t>Montagevorbereitung</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>WP</t>
+          <t>ALLE</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1718,12 +1718,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Förderantrag durch Kunden gestellt (Nachweis)</t>
+          <t>Anzahlung geschrieben</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>projektierer</t>
+          <t>buchhaltung</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1734,31 +1734,23 @@
       <c r="K26" t="inlineStr">
         <is>
           <t>keine</t>
-        </is>
-      </c>
-      <c r="N26" t="n">
-        <v>21</v>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>aktivierung</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>foerderung</t>
+          <t>montagevorbereitung</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Förderung</t>
+          <t>Montagevorbereitung</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>WP</t>
+          <t>ALLE</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1766,47 +1758,39 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Zusage liegt vor</t>
+          <t>Anzahlung bezahlt</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>projektierer</t>
+          <t>buchhaltung</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>J</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
           <t>keine</t>
-        </is>
-      </c>
-      <c r="N27" t="n">
-        <v>-1</v>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>montage</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>foerderung</t>
+          <t>montagevorbereitung</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Förderung</t>
+          <t>Montagevorbereitung</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>WP</t>
+          <t>ALLE</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1814,7 +1798,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>BnD nach Abnahme erstellt</t>
+          <t>Projekt zur Montage freigegeben</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Wächter für die Phase Montage.</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1830,26 +1819,18 @@
       <c r="K28" t="inlineStr">
         <is>
           <t>keine</t>
-        </is>
-      </c>
-      <c r="N28" t="n">
-        <v>10</v>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>montage</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>montagevorbereitung</t>
+          <t>abnahme_freigabe</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Montagevorbereitung</t>
+          <t>Abnahme &amp; Freigabe</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1862,17 +1843,22 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Anzahlung geschrieben</t>
+          <t>Montagebericht liegt vor</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>buchhaltung</t>
+          <t>projektierer</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
           <t>J</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>M+1</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -1884,12 +1870,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>montagevorbereitung</t>
+          <t>abnahme_freigabe</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Montagevorbereitung</t>
+          <t>Abnahme &amp; Freigabe</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1902,17 +1888,22 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Anzahlung bezahlt</t>
+          <t>Inbetriebnahmeprotokoll liegt vor</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>buchhaltung</t>
+          <t>projektierer</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
           <t>J</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>M+1</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -1924,12 +1915,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>montagevorbereitung</t>
+          <t>abnahme_freigabe</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Montagevorbereitung</t>
+          <t>Abnahme &amp; Freigabe</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1942,12 +1933,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Projekt zur Montage freigegeben</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Wächter für die Phase Montage.</t>
+          <t>Abnahmeprotokoll mit Kundenunterschrift</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1958,6 +1944,11 @@
       <c r="H31" t="inlineStr">
         <is>
           <t>J</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>M+1</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -1983,11 +1974,16 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Montagebericht liegt vor</t>
+          <t>Restarbeiten/Reklamationen erfasst</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Eigene Liste am Gewerk (Text, Foto, Verantwortlicher, Status).</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2002,7 +1998,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>M+1</t>
+          <t>M+3</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2028,16 +2024,16 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Inbetriebnahmeprotokoll liegt vor</t>
+          <t>Rechnung freigegeben</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>projektierer</t>
+          <t>buchhaltung</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2047,7 +2043,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>M+1</t>
+          <t>M+5</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2073,11 +2069,16 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Abnahmeprotokoll mit Kundenunterschrift</t>
+          <t>BnD nach Abnahme erstellt</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Bestätigung nach Durchführung (KfW) – nur bei gefördertem Auftrag, sonst auf „entfällt“ setzen.</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2092,42 +2093,43 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>M+1</t>
-        </is>
-      </c>
+          <t>M+10</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr">
         <is>
           <t>keine</t>
         </is>
       </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>abnahme_freigabe</t>
+          <t>pv_standard</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Abnahme &amp; Freigabe</t>
+          <t>PV Standard</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ALLE</t>
+          <t>PV</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Restarbeiten/Reklamationen erfasst</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>Eigene Liste am Gewerk (Text, Foto, Verantwortlicher, Status).</t>
+          <t>Feinplanung Dach/Strang/Speicherort</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2142,7 +2144,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>M+3</t>
+          <t>+14</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2154,30 +2156,30 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>abnahme_freigabe</t>
+          <t>pv_standard</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Abnahme &amp; Freigabe</t>
+          <t>PV Standard</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ALLE</t>
+          <t>PV</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Rechnung freigegeben</t>
+          <t>Netzanschlussbegehren beim Netzbetreiber</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>buchhaltung</t>
+          <t>elektroplaner</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -2187,7 +2189,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>M+5</t>
+          <t>FP+5</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2213,11 +2215,11 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Feinplanung Dach/Strang/Speicherort</t>
+          <t>Gerüst bestellen</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2232,7 +2234,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>+14</t>
+          <t>M-14</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2258,16 +2260,16 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Netzanschlussbegehren beim Netzbetreiber</t>
+          <t>Material bestellen</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>elektroplaner</t>
+          <t>projektierer</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2277,7 +2279,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>FP+5</t>
+          <t>FP+7</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2303,16 +2305,16 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Gerüst bestellen</t>
+          <t>Inbetriebnahme + Fertigmeldung Netzbetreiber</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>projektierer</t>
+          <t>elektroplaner</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2322,7 +2324,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>M-14</t>
+          <t>M+5</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2348,11 +2350,11 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Material bestellen</t>
+          <t>Marktstammdatenregister eingetragen</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2367,7 +2369,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>FP+7</t>
+          <t>M+20</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2379,25 +2381,25 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>pv_standard</t>
+          <t>wb_standard</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PV Standard</t>
+          <t>Wallbox Standard</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>PV</t>
+          <t>WB</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Inbetriebnahme + Fertigmeldung Netzbetreiber</t>
+          <t>Wallbox beim Netzbetreiber anmelden</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2412,7 +2414,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>M+5</t>
+          <t>+5</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -2424,25 +2426,25 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>pv_standard</t>
+          <t>wb_standard</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>PV Standard</t>
+          <t>Wallbox Standard</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>PV</t>
+          <t>WB</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Marktstammdatenregister eingetragen</t>
+          <t>Material bestellen</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2457,7 +2459,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>M+20</t>
+          <t>+7</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -2483,16 +2485,16 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Wallbox beim Netzbetreiber anmelden</t>
+          <t>Montage + Protokoll</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>elektroplaner</t>
+          <t>projektierer</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2502,7 +2504,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>+5</t>
+          <t>M+1</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -2514,25 +2516,25 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>wb_standard</t>
+          <t>kl_standard</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Wallbox Standard</t>
+          <t>Klima Standard</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>WB</t>
+          <t>KL</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Material bestellen</t>
+          <t>Feinplanung Innen-/Außengerät, Leitungsweg, Kondensat</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2547,7 +2549,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>+7</t>
+          <t>+14</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -2559,25 +2561,25 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>wb_standard</t>
+          <t>kl_standard</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Wallbox Standard</t>
+          <t>Klima Standard</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>WB</t>
+          <t>KL</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Montage + Protokoll</t>
+          <t>Material bestellen</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2592,7 +2594,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>M+1</t>
+          <t>FP+7</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -2618,11 +2620,11 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Feinplanung Innen-/Außengerät, Leitungsweg, Kondensat</t>
+          <t>Montage + Inbetriebnahme (Kältemittel-Nachweis)</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2637,100 +2639,10 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>+14</t>
+          <t>M+1</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
-        <is>
-          <t>keine</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>kl_standard</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Klima Standard</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>KL</t>
-        </is>
-      </c>
-      <c r="D47" t="n">
-        <v>2</v>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Material bestellen</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>projektierer</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>FP+7</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>keine</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>kl_standard</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Klima Standard</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>KL</t>
-        </is>
-      </c>
-      <c r="D48" t="n">
-        <v>3</v>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Montage + Inbetriebnahme (Kältemittel-Nachweis)</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>projektierer</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>M+1</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
         <is>
           <t>keine</t>
         </is>
@@ -2747,7 +2659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2889,7 +2801,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>WP</t>
+          <t>ALLE</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2899,7 +2811,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>foerderung</t>
+          <t>montagevorbereitung</t>
         </is>
       </c>
     </row>
@@ -2916,14 +2828,14 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>montagevorbereitung</t>
+          <t>abnahme_freigabe</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ALLE</t>
+          <t>PV</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2933,14 +2845,14 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>abnahme_freigabe</t>
+          <t>pv_standard</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PV</t>
+          <t>WB</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2950,14 +2862,14 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>pv_standard</t>
+          <t>wb_standard</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>WB</t>
+          <t>KL</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2966,23 +2878,6 @@
         </is>
       </c>
       <c r="C13" t="inlineStr">
-        <is>
-          <t>wb_standard</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>KL</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>IMMER</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
         <is>
           <t>kl_standard</t>
         </is>
@@ -5416,7 +5311,6 @@
           <t>J</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5449,7 +5343,6 @@
           <t>J</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5482,7 +5375,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5515,7 +5407,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5548,7 +5439,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -5581,7 +5471,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5614,7 +5503,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5647,7 +5535,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5680,7 +5567,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5713,7 +5599,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5746,7 +5631,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5779,7 +5663,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5812,7 +5695,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5845,7 +5727,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5878,7 +5759,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5948,7 +5828,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5981,7 +5860,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -6051,7 +5929,6 @@
           <t>J</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -6084,7 +5961,6 @@
           <t>J</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -6117,7 +5993,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -6150,7 +6025,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -6183,7 +6057,6 @@
           <t>J</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -6216,7 +6089,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6249,7 +6121,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6282,7 +6153,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6315,7 +6185,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -6348,7 +6217,6 @@
           <t>J</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -6381,7 +6249,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -6414,7 +6281,6 @@
           <t>J</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -6447,7 +6313,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -6480,7 +6345,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -6513,7 +6377,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -6546,7 +6409,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -6579,7 +6441,6 @@
           <t>J</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -6612,7 +6473,6 @@
           <t>J</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -6645,7 +6505,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -6678,7 +6537,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -6711,7 +6569,6 @@
           <t>J</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -6744,7 +6601,6 @@
           <t>J</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -6777,7 +6633,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -6847,7 +6702,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -6880,7 +6734,6 @@
           <t>J</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -6913,7 +6766,6 @@
           <t>J</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -6946,7 +6798,6 @@
           <t>J</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -6979,7 +6830,6 @@
           <t>J</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -7012,7 +6862,6 @@
           <t>J</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Abnahme & Freigabe: Pflicht-Schritt Abweichungen zum Angebot geprueft
Andreas 27.09.2026: neuer Schritt 5 (M+4, Pflicht) vor der Rechnungs-
freigabe; Rechnung freigegeben und BnD ruecken auf 6/7. Blatt validiert
(0 Fehler/0 Warnungen); Migration ergaenzt den Punkt an bestehenden
offenen Gewerken (4 lokal, idempotent, doppelt gelaufen); Suite 117/117.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projektierung_logik_v1.xlsx
+++ b/projektierung_logik_v1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P46"/>
+  <dimension ref="A1:P47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2028,12 +2028,17 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Rechnung freigegeben</t>
+          <t>Abweichungen zum Angebot geprüft, ggf. Nachtrag</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Mehr-/Minderleistungen aus der Montage mit dem Auftrag abgleichen, bevor die Rechnung freigegeben wird.</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>buchhaltung</t>
+          <t>projektierer</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2043,14 +2048,20 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>M+5</t>
-        </is>
-      </c>
+          <t>M+4</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr">
         <is>
           <t>keine</t>
         </is>
       </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2073,17 +2084,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>BnD nach Abnahme erstellt</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>Bestätigung nach Durchführung (KfW) – nur bei gefördertem Auftrag, sonst auf „entfällt“ setzen.</t>
+          <t>Rechnung freigegeben</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>projektierer</t>
+          <t>buchhaltung</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2093,43 +2099,42 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>M+10</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr"/>
+          <t>M+5</t>
+        </is>
+      </c>
       <c r="K34" t="inlineStr">
         <is>
           <t>keine</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>pv_standard</t>
+          <t>abnahme_freigabe</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PV Standard</t>
+          <t>Abnahme &amp; Freigabe</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>PV</t>
+          <t>ALLE</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Feinplanung Dach/Strang/Speicherort</t>
+          <t>BnD nach Abnahme erstellt</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Bestätigung nach Durchführung (KfW) – nur bei gefördertem Auftrag, sonst auf „entfällt“ setzen.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2144,7 +2149,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>+14</t>
+          <t>M+10</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2170,16 +2175,16 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Netzanschlussbegehren beim Netzbetreiber</t>
+          <t>Feinplanung Dach/Strang/Speicherort</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>elektroplaner</t>
+          <t>projektierer</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -2189,7 +2194,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>FP+5</t>
+          <t>+14</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2215,16 +2220,16 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Gerüst bestellen</t>
+          <t>Netzanschlussbegehren beim Netzbetreiber</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>projektierer</t>
+          <t>elektroplaner</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2234,7 +2239,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>M-14</t>
+          <t>FP+5</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2260,11 +2265,11 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Material bestellen</t>
+          <t>Gerüst bestellen</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2279,7 +2284,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>FP+7</t>
+          <t>M-14</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2305,16 +2310,16 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Inbetriebnahme + Fertigmeldung Netzbetreiber</t>
+          <t>Material bestellen</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>elektroplaner</t>
+          <t>projektierer</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2324,7 +2329,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>M+5</t>
+          <t>FP+7</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2350,16 +2355,16 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Marktstammdatenregister eingetragen</t>
+          <t>Inbetriebnahme + Fertigmeldung Netzbetreiber</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>projektierer</t>
+          <t>elektroplaner</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2369,7 +2374,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>M+20</t>
+          <t>M+5</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2381,30 +2386,30 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>wb_standard</t>
+          <t>pv_standard</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Wallbox Standard</t>
+          <t>PV Standard</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>WB</t>
+          <t>PV</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Wallbox beim Netzbetreiber anmelden</t>
+          <t>Marktstammdatenregister eingetragen</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>elektroplaner</t>
+          <t>projektierer</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2414,7 +2419,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>+5</t>
+          <t>M+20</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -2440,16 +2445,16 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Material bestellen</t>
+          <t>Wallbox beim Netzbetreiber anmelden</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>projektierer</t>
+          <t>elektroplaner</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2459,7 +2464,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>+7</t>
+          <t>+5</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -2485,11 +2490,11 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Montage + Protokoll</t>
+          <t>Material bestellen</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2504,7 +2509,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>M+1</t>
+          <t>+7</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -2516,25 +2521,25 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>kl_standard</t>
+          <t>wb_standard</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Klima Standard</t>
+          <t>Wallbox Standard</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>KL</t>
+          <t>WB</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Feinplanung Innen-/Außengerät, Leitungsweg, Kondensat</t>
+          <t>Montage + Protokoll</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2549,7 +2554,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>+14</t>
+          <t>M+1</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -2575,11 +2580,11 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Material bestellen</t>
+          <t>Feinplanung Innen-/Außengerät, Leitungsweg, Kondensat</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2594,7 +2599,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>FP+7</t>
+          <t>+14</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -2620,29 +2625,74 @@
         </is>
       </c>
       <c r="D46" t="n">
+        <v>2</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Material bestellen</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>projektierer</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>FP+7</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>keine</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>kl_standard</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Klima Standard</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>KL</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
         <v>3</v>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>Montage + Inbetriebnahme (Kältemittel-Nachweis)</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
+      <c r="G47" t="inlineStr">
         <is>
           <t>projektierer</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
         <is>
           <t>M+1</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
+      <c r="K47" t="inlineStr">
         <is>
           <t>keine</t>
         </is>

</xml_diff>

<commit_message>
PLAN_PROJ_V4 Phase 90: Kanban zweigeteilt, Abnahme/Freigabe getrennt, Vorlauf-Ampel, 15-Min-Takt, Aktionen ohne Seitensprung
- Board: Auftragseingang unterminiert | terminiert (Drop oeffnet Team + Termin), alle Spalten chronologisch
- Phasen abnahme + freigabe (Pakete, Waechter, Rechnung freigeben), Migration migration_abnahme_freigabe_split
- Vorlauf-Ampel je Gewerk (Parameter 8/4 Wochen) auf Karte, Liste, Chronologisch, Akte; Filter + Kachel
- 15-Minuten-Takt (step 900, serverseitige Rundung) inkl. Montage gestartet/fertig mit Uhrzeit
- Akte: Aufgaben-Aktionen per fetch (JSON, Partial _aufgabe.html), Scroll-Erhalt fuer alle uebrigen POSTs
- Tests tests/test_projektierung_v4.py

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projektierung_logik_v1.xlsx
+++ b/projektierung_logik_v1.xlsx
@@ -1825,12 +1825,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>abnahme_freigabe</t>
+          <t>abnahme</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Abnahme &amp; Freigabe</t>
+          <t>Abnahme</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1870,12 +1870,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>abnahme_freigabe</t>
+          <t>abnahme</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Abnahme &amp; Freigabe</t>
+          <t>Abnahme</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1915,12 +1915,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>abnahme_freigabe</t>
+          <t>abnahme</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Abnahme &amp; Freigabe</t>
+          <t>Abnahme</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1960,12 +1960,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>abnahme_freigabe</t>
+          <t>abnahme</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Abnahme &amp; Freigabe</t>
+          <t>Abnahme</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2010,12 +2010,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>abnahme_freigabe</t>
+          <t>abnahme</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Abnahme &amp; Freigabe</t>
+          <t>Abnahme</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2051,27 +2051,21 @@
           <t>M+4</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr">
         <is>
           <t>keine</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
-      <c r="P33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>abnahme_freigabe</t>
+          <t>freigabe</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Abnahme &amp; Freigabe</t>
+          <t>Freigabe</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2080,11 +2074,16 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
           <t>Rechnung freigegeben</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Wird über „Rechnung freigeben“ (Restarbeiten-Pflichtfrage) erledigt – Wechsel nach Abgeschlossen.</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2111,12 +2110,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>abnahme_freigabe</t>
+          <t>freigabe</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Abnahme &amp; Freigabe</t>
+          <t>Freigabe</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2125,7 +2124,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -2709,7 +2708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2878,14 +2877,14 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>abnahme_freigabe</t>
+          <t>abnahme</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PV</t>
+          <t>ALLE</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2895,14 +2894,14 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>pv_standard</t>
+          <t>freigabe</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>WB</t>
+          <t>PV</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2912,22 +2911,39 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>wb_standard</t>
+          <t>pv_standard</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>IMMER</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>wb_standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>KL</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>IMMER</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>kl_standard</t>
         </is>

</xml_diff>

<commit_message>
PLAN_PROJ_V4 Phase 91: Pakete umgebaut, Fit for Future Ja/Nein, FP-Fragen, Sub-Mails mit Restoel/Stemm/Erdarbeiten
- Auftragsunterlagen -> Planung WP Schritt 1 (PV/KL/WB: AE Schritt 5), Montageteam -> AE Schritt 2
- Fit for Future als Auswahl mit Steckbrief-Vorbelegung und Rueckschreiben, HEMS-IBN abhaengig
- FP-E05/FP-E06/FP-O04 (sichtbar_wenn), Steckbrief restoel_liter/stemmarbeiten/erdleitung_m
- Platzhalter {restoel} {stemmarbeiten} {erdarbeiten}, Vorlagen GaLa/Entsorgung ergaenzt
- Migration migration_pakete_v4; Erdleitung = Pos. 102 (Plan nannte 139/140, siehe Entscheidungen)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projektierung_logik_v1.xlsx
+++ b/projektierung_logik_v1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P47"/>
+  <dimension ref="A1:P48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,7 +531,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Auftragsunterlagen prüfen (Angebot, Protokoll, Fotos)</t>
+          <t>Kunde kontaktieren, Ablauf erklären, Feinplanungstermin abstimmen</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -546,11 +546,16 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>kalender</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>feinplanung</t>
         </is>
       </c>
       <c r="N2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -579,7 +584,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Kunde kontaktieren, Ablauf erklären, Feinplanungstermin abstimmen</t>
+          <t>Montageteam zuweisen</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Team + Termin (Montagetermin) – die Karte rutscht im Board in „Auftragseingang · terminiert“.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -599,15 +609,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>feinplanung</t>
-        </is>
-      </c>
-      <c r="N3" t="n">
-        <v>3</v>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>aktivierung</t>
+          <t>montage</t>
         </is>
       </c>
     </row>
@@ -720,30 +722,25 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>feinplanung_vot</t>
+          <t>auftragseingang</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Feinplanung VOT</t>
+          <t>Auftragseingang</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>WP</t>
+          <t>ALLE</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Feinplanungs-Erfassung durchführen</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Bis Phase 80 als Häkchen; danach Formular feinplanung_wp (vorbelegt aus der Vertriebs-Erfassung).</t>
+          <t>Auftragsunterlagen prüfen (Angebot, Protokoll, Fotos)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -758,20 +755,20 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>formular</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>feinplanung_wp</t>
+          <t>keine</t>
         </is>
       </c>
       <c r="N6" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
           <t>aktivierung</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>sparte:PV|KL|WB</t>
         </is>
       </c>
     </row>
@@ -792,16 +789,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Heizlastberechnung liegt vor</t>
+          <t>Feinplanungs-Erfassung durchführen</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Heizreport öffnen, Ergebnis-PDF in Galerie „Montagedokumente“ ablegen.</t>
+          <t>Bis Phase 80 als Häkchen; danach Formular feinplanung_wp (vorbelegt aus der Vertriebs-Erfassung).</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -816,20 +813,20 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>api</t>
+          <t>formular</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>heizreport</t>
+          <t>feinplanung_wp</t>
         </is>
       </c>
       <c r="N7" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>feinplanung</t>
+          <t>aktivierung</t>
         </is>
       </c>
     </row>
@@ -850,40 +847,40 @@
         </is>
       </c>
       <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Heizlastberechnung liegt vor</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Heizreport öffnen, Ergebnis-PDF in Galerie „Montagedokumente“ ablegen.</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>projektierer</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>api</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>heizreport</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
         <v>3</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Fotos abgelegt (Alte Heizung, Elektro, Außengerät, Allgemein)</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Häkchen setzt sich automatisch, sobald in allen vier Ordnern mindestens ein Bild liegt.</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>projektierer</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>galerie</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>Alte Heizung|Elektro|Außengerät|Allgemein</t>
-        </is>
-      </c>
-      <c r="N8" t="n">
-        <v>1</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -908,11 +905,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Abweichungen zum Angebot geprüft, ggf. Nachtrag</t>
+          <t>Fotos abgelegt (Alte Heizung, Elektro, Außengerät, Allgemein)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Häkchen setzt sich automatisch, sobald in allen vier Ordnern mindestens ein Bild liegt.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -927,11 +929,16 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>galerie</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Alte Heizung|Elektro|Außengerät|Allgemein</t>
         </is>
       </c>
       <c r="N9" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -956,11 +963,11 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Gerät/Paket final festgelegt (Steckbrief)</t>
+          <t>Abweichungen zum Angebot geprüft, ggf. Nachtrag</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -990,12 +997,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>planung_wp</t>
+          <t>feinplanung_vot</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Planung WP</t>
+          <t>Feinplanung VOT</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1004,11 +1011,11 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Montageteam zuweisen</t>
+          <t>Gerät/Paket final festgelegt (Steckbrief)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1023,12 +1030,15 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>kalender</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>montage</t>
+          <t>keine</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>5</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>feinplanung</t>
         </is>
       </c>
     </row>
@@ -1049,36 +1059,34 @@
         </is>
       </c>
       <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Auftragsunterlagen prüfen (Angebot, Protokoll, Fotos)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>projektierer</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>keine</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
         <v>2</v>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Stückliste geprüft und Material bestellt</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>UGL-Bestellung Collin (Phase 80); AB des Großhändlers in Galerie „Montagedokumente“ ablegen.</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>projektierer</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>api</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>ugl_collin</t>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>aktivierung</t>
         </is>
       </c>
     </row>
@@ -1099,11 +1107,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>GaLa-Beauftragung (Fundament)</t>
+          <t>Stückliste geprüft und Material bestellt</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>UGL-Bestellung Collin (Phase 80); AB des Großhändlers in Galerie „Montagedokumente“ ablegen.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1118,17 +1131,12 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>auswahl</t>
+          <t>api</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>mail:GaLa-Bau@Außengerät</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>erfolgt bauseits | nicht erforderlich | beauftragt*</t>
+          <t>ugl_collin</t>
         </is>
       </c>
     </row>
@@ -1149,11 +1157,11 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>WP-Montage Sub beauftragen</t>
+          <t>GaLa-Beauftragung (Fundament + Erdarbeiten)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1173,12 +1181,12 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>mail:WP-Montage@Alte Heizung</t>
+          <t>mail:GaLa-Bau@Außengerät</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Montage durch Friondo* | Sub beauftragt*</t>
+          <t>erfolgt bauseits | nicht erforderlich | beauftragt*</t>
         </is>
       </c>
     </row>
@@ -1199,11 +1207,11 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Öltank-Entsorgung</t>
+          <t>WP-Montage Sub beauftragen</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1223,12 +1231,12 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>mail:Entsorgung@Öl-Tank</t>
+          <t>mail:WP-Montage@Alte Heizung</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>erfolgt bauseits | nicht erforderlich | beauftragt*</t>
+          <t>Montage durch Friondo* | Sub beauftragt*</t>
         </is>
       </c>
     </row>
@@ -1249,11 +1257,11 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Folierung geplant</t>
+          <t>Öltank-Entsorgung</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1271,44 +1279,44 @@
           <t>auswahl</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>mail:Entsorgung@Öl-Tank</t>
+        </is>
+      </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>keine Folierung | geplant*</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>steckbrief:folierung=ja</t>
+          <t>erfolgt bauseits | nicht erforderlich | beauftragt*</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>planung_elektro</t>
+          <t>planung_wp</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Planung Elektro</t>
+          <t>Planung WP</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ALLE</t>
+          <t>WP</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Elektro-Montageteam zuweisen</t>
+          <t>Folierung geplant</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>elektroplaner</t>
+          <t>projektierer</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1318,12 +1326,17 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>kalender</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>montage</t>
+          <t>auswahl</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>keine Folierung | geplant*</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>steckbrief:folierung=ja</t>
         </is>
       </c>
     </row>
@@ -1344,16 +1357,11 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Zählerschrank/Unterverteilung mit Auftrag bewertet</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Steckbrief-Feld Zählerschrank pflegen.</t>
+          <t>Elektro-Montageteam zuweisen</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1368,7 +1376,12 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>kalender</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>montage</t>
         </is>
       </c>
     </row>
@@ -1389,11 +1402,16 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Elektro-Sub</t>
+          <t>Zählerschrank/Unterverteilung mit Auftrag bewertet</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Steckbrief-Feld Zählerschrank pflegen.</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1408,17 +1426,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>auswahl</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>mail:Elektro@Elektro</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>erfolgt über Friondo* | erfolgt bauseits | Sub beauftragt*</t>
+          <t>keine</t>
         </is>
       </c>
     </row>
@@ -1439,16 +1447,11 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Netzbetreiber-Anmeldung WP (§14a) eingereicht</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Frist wird später nachgetragen.</t>
+          <t>Elektro-Sub</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1463,7 +1466,17 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>auswahl</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>mail:Elektro@Elektro</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>erfolgt über Friondo* | erfolgt bauseits | Sub beauftragt*</t>
         </is>
       </c>
     </row>
@@ -1484,11 +1497,11 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Zustimmung Netzbetreiber liegt vor</t>
+          <t>Netzbetreiber-Anmeldung WP (§14a) eingereicht</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1515,30 +1528,35 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>fit_for_future</t>
+          <t>planung_elektro</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Friondo Fit for Future</t>
+          <t>Planung Elektro</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>WP</t>
+          <t>ALLE</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Friondo HEMS geplant</t>
+          <t>Zustimmung Netzbetreiber liegt vor</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Frist wird später nachgetragen.</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>projektierer</t>
+          <t>elektroplaner</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1548,12 +1566,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>auswahl</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>Ja* | Nein*</t>
+          <t>keine</t>
         </is>
       </c>
     </row>
@@ -1574,16 +1587,16 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Friondo iMSys geplant</t>
+          <t>Friondo HEMS geplant</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>SpotmyEnergy-Portal; Zählerwechseltermin am Gewerk pflegen (Marker im Kalender).</t>
+          <t>Vorbelegt aus dem Steckbrief (hems) – mit „Übernehmen“ bestätigen.</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1598,12 +1611,17 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>link</t>
+          <t>auswahl</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>param:url_spotmyenergy</t>
+          <t>steckbrief:hems</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Ja* | Nein*</t>
         </is>
       </c>
     </row>
@@ -1624,11 +1642,16 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Friondo SpotDynamic</t>
+          <t>Friondo iMSys geplant</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>SpotmyEnergy-Portal; Zählerwechseltermin am Gewerk pflegen (Marker im Kalender).</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1643,12 +1666,17 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>link</t>
+          <t>auswahl</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>param:url_spotmyenergy</t>
+          <t>param:url_spotmyenergy;steckbrief:imsys</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Ja* | Nein*</t>
         </is>
       </c>
     </row>
@@ -1669,11 +1697,16 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>HEMS-Inbetriebnahme terminiert</t>
+          <t>Friondo SpotDynamic</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>SpotmyEnergy-Portal; vorbelegt aus dem Steckbrief (Dynamischer Tarif).</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1688,42 +1721,52 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>kalender</t>
+          <t>auswahl</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>sonstige</t>
+          <t>param:url_spotmyenergy;steckbrief:dyn_tarif</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Ja* | Nein*</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>montagevorbereitung</t>
+          <t>fit_for_future</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Montagevorbereitung</t>
+          <t>Friondo Fit for Future</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ALLE</t>
+          <t>WP</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Anzahlung geschrieben</t>
+          <t>HEMS-Inbetriebnahme terminiert</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Nur bei HEMS = Ja (sonst „entfällt“ automatisch).</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>buchhaltung</t>
+          <t>projektierer</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1733,7 +1776,17 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>kalender</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>sonstige</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>fit_for_future.1=Ja</t>
         </is>
       </c>
     </row>
@@ -1754,11 +1807,11 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Anzahlung bezahlt</t>
+          <t>Anzahlung geschrieben</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1794,21 +1847,16 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Projekt zur Montage freigegeben</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Wächter für die Phase Montage.</t>
+          <t>Anzahlung bezahlt</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>projektierer</t>
+          <t>buchhaltung</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1825,12 +1873,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>abnahme</t>
+          <t>montagevorbereitung</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Abnahme</t>
+          <t>Montagevorbereitung</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1839,11 +1887,16 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Montagebericht liegt vor</t>
+          <t>Projekt zur Montage freigegeben</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Wächter für die Phase Montage.</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1854,11 +1907,6 @@
       <c r="H29" t="inlineStr">
         <is>
           <t>J</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>M+1</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -1884,11 +1932,11 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Inbetriebnahmeprotokoll liegt vor</t>
+          <t>Montagebericht liegt vor</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1929,11 +1977,11 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Abnahmeprotokoll mit Kundenunterschrift</t>
+          <t>Inbetriebnahmeprotokoll liegt vor</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1974,16 +2022,11 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Restarbeiten/Reklamationen erfasst</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>Eigene Liste am Gewerk (Text, Foto, Verantwortlicher, Status).</t>
+          <t>Abnahmeprotokoll mit Kundenunterschrift</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1998,7 +2041,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>M+3</t>
+          <t>M+1</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2024,16 +2067,16 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Abweichungen zum Angebot geprüft, ggf. Nachtrag</t>
+          <t>Restarbeiten/Reklamationen erfasst</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Mehr-/Minderleistungen aus der Montage mit dem Auftrag abgleichen, bevor die Rechnung freigegeben wird.</t>
+          <t>Eigene Liste am Gewerk (Text, Foto, Verantwortlicher, Status).</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2048,7 +2091,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>M+4</t>
+          <t>M+3</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2060,12 +2103,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>freigabe</t>
+          <t>abnahme</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Freigabe</t>
+          <t>Abnahme</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2074,21 +2117,21 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Rechnung freigegeben</t>
+          <t>Abweichungen zum Angebot geprüft, ggf. Nachtrag</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Wird über „Rechnung freigeben“ (Restarbeiten-Pflichtfrage) erledigt – Wechsel nach Abgeschlossen.</t>
+          <t>Mehr-/Minderleistungen aus der Montage mit dem Auftrag abgleichen, bevor die Rechnung freigegeben wird.</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>buchhaltung</t>
+          <t>projektierer</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2098,7 +2141,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>M+5</t>
+          <t>M+4</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2124,21 +2167,21 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>BnD nach Abnahme erstellt</t>
+          <t>Rechnung freigegeben</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Bestätigung nach Durchführung (KfW) – nur bei gefördertem Auftrag, sonst auf „entfällt“ setzen.</t>
+          <t>Wird über „Rechnung freigeben“ (Restarbeiten-Pflichtfrage) erledigt – Wechsel nach Abgeschlossen.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>projektierer</t>
+          <t>buchhaltung</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2148,7 +2191,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>M+10</t>
+          <t>M+5</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2160,25 +2203,30 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>pv_standard</t>
+          <t>freigabe</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PV Standard</t>
+          <t>Freigabe</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>PV</t>
+          <t>ALLE</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Feinplanung Dach/Strang/Speicherort</t>
+          <t>BnD nach Abnahme erstellt</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Bestätigung nach Durchführung (KfW) – nur bei gefördertem Auftrag, sonst auf „entfällt“ setzen.</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2193,7 +2241,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>+14</t>
+          <t>M+10</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2219,16 +2267,16 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Netzanschlussbegehren beim Netzbetreiber</t>
+          <t>Feinplanung Dach/Strang/Speicherort</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>elektroplaner</t>
+          <t>projektierer</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2238,7 +2286,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>FP+5</t>
+          <t>+14</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2264,16 +2312,16 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Gerüst bestellen</t>
+          <t>Netzanschlussbegehren beim Netzbetreiber</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>projektierer</t>
+          <t>elektroplaner</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2283,7 +2331,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>M-14</t>
+          <t>FP+5</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2309,11 +2357,11 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Material bestellen</t>
+          <t>Gerüst bestellen</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2328,7 +2376,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>FP+7</t>
+          <t>M-14</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2354,16 +2402,16 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Inbetriebnahme + Fertigmeldung Netzbetreiber</t>
+          <t>Material bestellen</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>elektroplaner</t>
+          <t>projektierer</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2373,7 +2421,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>M+5</t>
+          <t>FP+7</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2399,16 +2447,16 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Marktstammdatenregister eingetragen</t>
+          <t>Inbetriebnahme + Fertigmeldung Netzbetreiber</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>projektierer</t>
+          <t>elektroplaner</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2418,7 +2466,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>M+20</t>
+          <t>M+5</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -2430,30 +2478,30 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>wb_standard</t>
+          <t>pv_standard</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Wallbox Standard</t>
+          <t>PV Standard</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>WB</t>
+          <t>PV</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Wallbox beim Netzbetreiber anmelden</t>
+          <t>Marktstammdatenregister eingetragen</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>elektroplaner</t>
+          <t>projektierer</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2463,7 +2511,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>+5</t>
+          <t>M+20</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -2489,16 +2537,16 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Material bestellen</t>
+          <t>Wallbox beim Netzbetreiber anmelden</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>projektierer</t>
+          <t>elektroplaner</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2508,7 +2556,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>+7</t>
+          <t>+5</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -2534,11 +2582,11 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Montage + Protokoll</t>
+          <t>Material bestellen</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2553,7 +2601,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>M+1</t>
+          <t>+7</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -2565,25 +2613,25 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>kl_standard</t>
+          <t>wb_standard</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Klima Standard</t>
+          <t>Wallbox Standard</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>KL</t>
+          <t>WB</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Feinplanung Innen-/Außengerät, Leitungsweg, Kondensat</t>
+          <t>Montage + Protokoll</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2598,7 +2646,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>+14</t>
+          <t>M+1</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -2624,11 +2672,11 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Material bestellen</t>
+          <t>Feinplanung Innen-/Außengerät, Leitungsweg, Kondensat</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2643,7 +2691,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>FP+7</t>
+          <t>+14</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -2669,29 +2717,74 @@
         </is>
       </c>
       <c r="D47" t="n">
+        <v>2</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Material bestellen</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>projektierer</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>FP+7</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>keine</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>kl_standard</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Klima Standard</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>KL</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
         <v>3</v>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E48" t="inlineStr">
         <is>
           <t>Montage + Inbetriebnahme (Kältemittel-Nachweis)</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
+      <c r="G48" t="inlineStr">
         <is>
           <t>projektierer</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
         <is>
           <t>M+1</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr">
+      <c r="K48" t="inlineStr">
         <is>
           <t>keine</t>
         </is>
@@ -3274,6 +3367,9 @@
 Gerät: {geraet}
 Außengerät/Aufstellung: {aussengeraet_details}
 Gewünschte Fertigstellung: vor dem Montagetermin {montagetermin}
+Erdarbeiten:
+{erdarbeiten}
+Fundament/Aufstellung (Maße siehe Steckbrief): {aussengeraet_details}
 {bemerkung}
 Fotos vom Aufstellort hängen an.
 Bei Rückfragen erreichen Sie uns unter den bekannten Kontaktdaten.
@@ -3395,7 +3491,9 @@
 Kunde: {kunde}
 Ausführungsadresse: {ausfuehrungsadresse}
 Telefon Kunde: {telefon_kunde}
-Öltank: {oeltank}
+Öltank (Größe · Material/Zugang): {oeltank}
+{restoel}
+{stemmarbeiten}
 Gewünschte Ausführung: vor dem Montagetermin {montagetermin}
 {bemerkung}
 Fotos vom Tankraum hängen an.
@@ -3428,7 +3526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3467,6 +3565,11 @@
           <t>vorbelegung_aus</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>sichtbar_wenn</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3776,17 +3879,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Öltank &amp; Hydraulik</t>
+          <t>Elektro</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>FP-O01</t>
+          <t>FP-E05</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Öltank vorhanden (Entsorgung)</t>
+          <t>Friondo iMSys gewünscht</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -3801,39 +3904,39 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>A07</t>
+          <t>P02</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Öltank &amp; Hydraulik</t>
+          <t>Elektro</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>FP-O02</t>
+          <t>FP-E06</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Öltank: Größe (Liter)</t>
+          <t>Friondo HEMS gewünscht</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>ja_nein</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>J</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>A09</t>
+          <t>P01</t>
         </is>
       </c>
     </row>
@@ -3845,27 +3948,27 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>FP-O03</t>
+          <t>FP-O01</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Öltank: Material/Zugang</t>
+          <t>Öltank vorhanden (Entsorgung)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>ja_nein</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>J</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>A08</t>
+          <t>A07</t>
         </is>
       </c>
     </row>
@@ -3877,12 +3980,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>FP-H01</t>
+          <t>FP-O02</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Hydraulik-Besonderheiten</t>
+          <t>Öltank: Größe (Liter)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -3893,6 +3996,11 @@
       <c r="F15" t="inlineStr">
         <is>
           <t>N</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>A09</t>
         </is>
       </c>
     </row>
@@ -3904,39 +4012,44 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>FP-H02</t>
+          <t>FP-O03</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Folierung gewünscht</t>
+          <t>Öltank: Material/Zugang</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>ja_nein</t>
+          <t>text</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>A08</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Heizlast</t>
+          <t>Öltank &amp; Hydraulik</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>FP-L01</t>
+          <t>FP-O04</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Heizlast (kW)</t>
+          <t>Restöl im Tank (Liter, geschätzt)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -3947,36 +4060,122 @@
       <c r="F17" t="inlineStr">
         <is>
           <t>J</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>FP-O01=Ja</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>Öltank &amp; Hydraulik</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>FP-H01</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Hydraulik-Besonderheiten</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Öltank &amp; Hydraulik</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>FP-H02</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Folierung gewünscht</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>Heizlast</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>FP-L01</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Heizlast (kW)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>zahl</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Heizlast</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
         <is>
           <t>FP-L02</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>Heizlast-Quelle</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>auswahl</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>Heizreport | Verbrauch | Schätzung</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>J</t>
         </is>
@@ -3993,7 +4192,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4249,7 +4448,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>hersteller</t>
+          <t>imsys</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -4259,24 +4458,24 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>position</t>
+          <t>fp_frage</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>030/031/045-056</t>
+          <t>FP-E05</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Ja→ja | Nein→nein</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>leistungsklasse</t>
+          <t>hems</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -4286,24 +4485,24 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>position</t>
+          <t>fp_frage</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>030/031</t>
+          <t>FP-E06</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>15 kW (Serie CS8800i)</t>
+          <t>Ja→ja | Nein→nein</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>leistungsklasse</t>
+          <t>restoel_liter</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -4313,24 +4512,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>position</t>
+          <t>fp_frage</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>045/050</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>4 kW (CS3800i)</t>
+          <t>FP-O04</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>leistungsklasse</t>
+          <t>hersteller</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -4345,12 +4539,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>046/051</t>
+          <t>030/031/045-056</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>6 kW (CS3800i)</t>
+          <t>Bosch</t>
         </is>
       </c>
     </row>
@@ -4372,12 +4566,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>047/052</t>
+          <t>030/031</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>7 kW (CS3800i)</t>
+          <t>15 kW (Serie CS8800i)</t>
         </is>
       </c>
     </row>
@@ -4399,12 +4593,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>048/053</t>
+          <t>045/050</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>10 kW (CS3800i)</t>
+          <t>4 kW (CS3800i)</t>
         </is>
       </c>
     </row>
@@ -4426,19 +4620,19 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>049/054</t>
+          <t>046/051</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>13 kW (CS3800i)</t>
+          <t>6 kW (CS3800i)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>innengeraet</t>
+          <t>leistungsklasse</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -4453,19 +4647,19 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>055</t>
+          <t>047/052</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>AWMB (integrierter 70-l-Puffer)</t>
+          <t>7 kW (CS3800i)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>innengeraet</t>
+          <t>leistungsklasse</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -4480,19 +4674,19 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>056</t>
+          <t>048/053</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>AWE + externer Puffer</t>
+          <t>10 kW (CS3800i)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>innengeraet</t>
+          <t>leistungsklasse</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -4507,12 +4701,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>045-049</t>
+          <t>049/054</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>AWM (Warmwasserspeicher 180 l integriert)</t>
+          <t>13 kW (CS3800i)</t>
         </is>
       </c>
     </row>
@@ -4534,19 +4728,19 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>050-054</t>
+          <t>055</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>AWE</t>
+          <t>AWMB (integrierter 70-l-Puffer)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>warmwasser</t>
+          <t>innengeraet</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -4561,19 +4755,19 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>069</t>
+          <t>056</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>390-l-Solarspeicher (bivalent, Solarthermie-Uebernahme)</t>
+          <t>AWE + externer Puffer</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>warmwasser</t>
+          <t>innengeraet</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4588,19 +4782,19 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>065</t>
+          <t>045-049</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>300-l-Warmwasserspeicher</t>
+          <t>AWM (Warmwasserspeicher 180 l integriert)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>warmwasser</t>
+          <t>innengeraet</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4610,24 +4804,24 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>frage</t>
+          <t>position</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>N02</t>
+          <t>050-054</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Nein→ohne Warmwasser | Ja→ueber die Waermepumpe</t>
+          <t>AWE</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>aufstellort</t>
+          <t>warmwasser</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -4642,19 +4836,19 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>010</t>
+          <t>069</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Boden (Fundament wird erstellt)</t>
+          <t>390-l-Solarspeicher (bivalent, Solarthermie-Uebernahme)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>aufstellort</t>
+          <t>warmwasser</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -4669,19 +4863,19 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>132</t>
+          <t>065</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Garagendach (Bodenkonsole)</t>
+          <t>300-l-Warmwasserspeicher</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>aufstellort</t>
+          <t>warmwasser</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4696,14 +4890,19 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>N04</t>
+          <t>N02</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Nein→ohne Warmwasser | Ja→ueber die Waermepumpe</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>zaehlerschrank</t>
+          <t>aufstellort</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -4713,24 +4912,24 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>frage</t>
+          <t>position</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>E03</t>
+          <t>010</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2-Feld→wird erneuert: Zweifeld | 3-Feld→wird erneuert: Dreifeld | 4-Feld und mehr→wird erneuert: Vierfeld</t>
+          <t>Boden (Fundament wird erstellt)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>zaehlerschrank</t>
+          <t>aufstellort</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -4745,19 +4944,19 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>152</t>
+          <t>132</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>bleibt · Unterverteilung wird gesetzt</t>
+          <t>Garagendach (Bodenkonsole)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>zaehlerschrank</t>
+          <t>aufstellort</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -4772,19 +4971,14 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>E02</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Nein→bleibt</t>
+          <t>N04</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>oeltank</t>
+          <t>zaehlerschrank</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -4799,19 +4993,19 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>A07</t>
+          <t>E03</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Nein→nein | Ja→ja</t>
+          <t>2-Feld→wird erneuert: Zweifeld | 3-Feld→wird erneuert: Dreifeld | 4-Feld und mehr→wird erneuert: Vierfeld</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>oeltank_groesse</t>
+          <t>zaehlerschrank</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -4821,19 +5015,24 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>frage</t>
+          <t>position</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>A09</t>
+          <t>152</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>bleibt · Unterverteilung wird gesetzt</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>oeltank_groesse</t>
+          <t>zaehlerschrank</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -4848,14 +5047,19 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>A19</t>
+          <t>E02</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Nein→bleibt</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>oeltank_material</t>
+          <t>oeltank</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4870,14 +5074,19 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>A08</t>
+          <t>A07</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Nein→nein | Ja→ja</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>alte_anlage</t>
+          <t>oeltank_groesse</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4892,14 +5101,14 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>A01</t>
+          <t>A09</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>alte_anlage_standort</t>
+          <t>oeltank_groesse</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4914,19 +5123,14 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>A04</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>DG→Dachzentrale (DG) | *→</t>
+          <t>A19</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>hems</t>
+          <t>oeltank_material</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4941,19 +5145,14 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>P01</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Ja→ja | Nein→nein</t>
+          <t>A08</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>imsys</t>
+          <t>alte_anlage</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -4968,19 +5167,14 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>P02</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Ja→ja | Nein→nein</t>
+          <t>A01</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>dyn_tarif</t>
+          <t>alte_anlage_standort</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4995,19 +5189,19 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>P03</t>
+          <t>A04</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Ja→ja | Nein→nein</t>
+          <t>DG→Dachzentrale (DG) | *→</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>kran</t>
+          <t>hems</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -5022,19 +5216,19 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>N09</t>
+          <t>P01</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Ja→Mobiler Kran eingeplant | Nein→nicht erforderlich</t>
+          <t>Ja→ja | Nein→nein</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>kran</t>
+          <t>imsys</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -5044,24 +5238,24 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>position</t>
+          <t>frage</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>135</t>
+          <t>P02</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Kran als Eventualposition im Angebot</t>
+          <t>Ja→ja | Nein→nein</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>besonderheiten</t>
+          <t>dyn_tarif</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -5071,24 +5265,24 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>position</t>
+          <t>frage</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Z24</t>
+          <t>P03</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Solarthermie wird stillgelegt (Z24)</t>
+          <t>Ja→ja | Nein→nein</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>besonderheiten</t>
+          <t>kran</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -5103,29 +5297,240 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>A12</t>
+          <t>N09</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Ja→Mobiler Kran eingeplant | Nein→nicht erforderlich</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>kran</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>135</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Kran als Eventualposition im Angebot</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>besonderheiten</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Z24</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Solarthermie wird stillgelegt (Z24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>besonderheiten</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>frage</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>A12</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
           <t>dach</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>PV</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>frage</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>PV01</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>stemmarbeiten</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>126</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>ja (Pos. 126, Menge {menge})</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>stemmarbeiten</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>frage</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>A16</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Ja→ja (laut Erfassung) | Nein→nein</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>stemmarbeiten</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>fest</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>erdleitung_m</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>102</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>{menge} m (Pos. 102 Erdleitung)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>erdleitung_m</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>frage</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>A05</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>*→{wert} m (laut Erfassung)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
PLAN_PROJ_V4 Phase 92: BzA erfassen, Kundenmail BzA, KfW-Felder
- Gewerk-Felder bza_id/bza_erstellt_am/bza_gesendet_am/bza_datei_id/kfw_antragsnummer/kfw_zusage_am
- Aufgabe BzA mit Portal/Datenblatt/BzA erfassen (nur gefoerdert, sonst entfaellt), PDF in Galerie Foerderung
- Kundenmail BzA (Vorlage in der Parametrierung, Vorschau mit Bearbeiten, Demo-Testadresse)
- KfW-Antragsnummer/Zusage als nicht verpflichtende Aufgabe (Montagevorbereitung), Anzeige in Steckbrief/PDF/Datenblatt
- Migration migration_bza_v4

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projektierung_logik_v1.xlsx
+++ b/projektierung_logik_v1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P48"/>
+  <dimension ref="A1:P49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -682,12 +682,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BzA erstellen und versenden</t>
+          <t>BzA erstellen und an Kunden senden</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>BzA-Portal öffnen; Datenblatt mit Kopier-Buttons folgt (Phase 80).</t>
+          <t>BzA-Portal ↗ · Datenblatt (Kopier-Buttons) · BzA erfassen (ID, Datum, PDF → Galerie „Förderung“) → Kundenmail „BzA“. Nur bei gefördertem Auftrag, sonst „entfällt (nicht gefördert)“.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -702,12 +702,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>param:url_bza_portal</t>
+          <t>bza</t>
         </is>
       </c>
       <c r="N5" t="n">
@@ -1918,12 +1913,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>abnahme</t>
+          <t>montagevorbereitung</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Abnahme</t>
+          <t>Montagevorbereitung</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1932,11 +1927,16 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Montagebericht liegt vor</t>
+          <t>KfW-Antragsnummer/Zusage eingetragen</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Antragsnummer und Zusage-Datum der KfW eintragen (kein Wächter – Frist folgt).</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1946,17 +1946,17 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>M+1</t>
+          <t>N</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>keine</t>
+          <t>bza</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>kfw</t>
         </is>
       </c>
     </row>
@@ -1977,11 +1977,11 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Inbetriebnahmeprotokoll liegt vor</t>
+          <t>Montagebericht liegt vor</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2022,11 +2022,11 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Abnahmeprotokoll mit Kundenunterschrift</t>
+          <t>Inbetriebnahmeprotokoll liegt vor</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2067,16 +2067,11 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Restarbeiten/Reklamationen erfasst</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Eigene Liste am Gewerk (Text, Foto, Verantwortlicher, Status).</t>
+          <t>Abnahmeprotokoll mit Kundenunterschrift</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2091,7 +2086,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>M+3</t>
+          <t>M+1</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2117,16 +2112,16 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Abweichungen zum Angebot geprüft, ggf. Nachtrag</t>
+          <t>Restarbeiten/Reklamationen erfasst</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Mehr-/Minderleistungen aus der Montage mit dem Auftrag abgleichen, bevor die Rechnung freigegeben wird.</t>
+          <t>Eigene Liste am Gewerk (Text, Foto, Verantwortlicher, Status).</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2141,7 +2136,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>M+4</t>
+          <t>M+3</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2153,12 +2148,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>freigabe</t>
+          <t>abnahme</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Freigabe</t>
+          <t>Abnahme</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2167,21 +2162,21 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Rechnung freigegeben</t>
+          <t>Abweichungen zum Angebot geprüft, ggf. Nachtrag</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Wird über „Rechnung freigeben“ (Restarbeiten-Pflichtfrage) erledigt – Wechsel nach Abgeschlossen.</t>
+          <t>Mehr-/Minderleistungen aus der Montage mit dem Auftrag abgleichen, bevor die Rechnung freigegeben wird.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>buchhaltung</t>
+          <t>projektierer</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2191,7 +2186,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>M+5</t>
+          <t>M+4</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2217,21 +2212,21 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>BnD nach Abnahme erstellt</t>
+          <t>Rechnung freigegeben</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Bestätigung nach Durchführung (KfW) – nur bei gefördertem Auftrag, sonst auf „entfällt“ setzen.</t>
+          <t>Wird über „Rechnung freigeben“ (Restarbeiten-Pflichtfrage) erledigt – Wechsel nach Abgeschlossen.</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>projektierer</t>
+          <t>buchhaltung</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -2241,7 +2236,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>M+10</t>
+          <t>M+5</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2253,25 +2248,30 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>pv_standard</t>
+          <t>freigabe</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PV Standard</t>
+          <t>Freigabe</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>PV</t>
+          <t>ALLE</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Feinplanung Dach/Strang/Speicherort</t>
+          <t>BnD nach Abnahme erstellt</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Bestätigung nach Durchführung (KfW) – nur bei gefördertem Auftrag, sonst auf „entfällt“ setzen.</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2286,7 +2286,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>+14</t>
+          <t>M+10</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2312,16 +2312,16 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Netzanschlussbegehren beim Netzbetreiber</t>
+          <t>Feinplanung Dach/Strang/Speicherort</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>elektroplaner</t>
+          <t>projektierer</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2331,7 +2331,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>FP+5</t>
+          <t>+14</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2357,16 +2357,16 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Gerüst bestellen</t>
+          <t>Netzanschlussbegehren beim Netzbetreiber</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>projektierer</t>
+          <t>elektroplaner</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2376,7 +2376,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>M-14</t>
+          <t>FP+5</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2402,11 +2402,11 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Material bestellen</t>
+          <t>Gerüst bestellen</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2421,7 +2421,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>FP+7</t>
+          <t>M-14</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2447,16 +2447,16 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Inbetriebnahme + Fertigmeldung Netzbetreiber</t>
+          <t>Material bestellen</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>elektroplaner</t>
+          <t>projektierer</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>M+5</t>
+          <t>FP+7</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -2492,16 +2492,16 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Marktstammdatenregister eingetragen</t>
+          <t>Inbetriebnahme + Fertigmeldung Netzbetreiber</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>projektierer</t>
+          <t>elektroplaner</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2511,7 +2511,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>M+20</t>
+          <t>M+5</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -2523,30 +2523,30 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>wb_standard</t>
+          <t>pv_standard</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Wallbox Standard</t>
+          <t>PV Standard</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>WB</t>
+          <t>PV</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Wallbox beim Netzbetreiber anmelden</t>
+          <t>Marktstammdatenregister eingetragen</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>elektroplaner</t>
+          <t>projektierer</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2556,7 +2556,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>+5</t>
+          <t>M+20</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -2582,16 +2582,16 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Material bestellen</t>
+          <t>Wallbox beim Netzbetreiber anmelden</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>projektierer</t>
+          <t>elektroplaner</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2601,7 +2601,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>+7</t>
+          <t>+5</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -2627,11 +2627,11 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Montage + Protokoll</t>
+          <t>Material bestellen</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2646,7 +2646,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>M+1</t>
+          <t>+7</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -2658,25 +2658,25 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>kl_standard</t>
+          <t>wb_standard</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Klima Standard</t>
+          <t>Wallbox Standard</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>KL</t>
+          <t>WB</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Feinplanung Innen-/Außengerät, Leitungsweg, Kondensat</t>
+          <t>Montage + Protokoll</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>+14</t>
+          <t>M+1</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -2717,11 +2717,11 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Material bestellen</t>
+          <t>Feinplanung Innen-/Außengerät, Leitungsweg, Kondensat</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>FP+7</t>
+          <t>+14</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -2762,29 +2762,74 @@
         </is>
       </c>
       <c r="D48" t="n">
+        <v>2</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Material bestellen</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>projektierer</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>FP+7</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>keine</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>kl_standard</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Klima Standard</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>KL</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
         <v>3</v>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t>Montage + Inbetriebnahme (Kältemittel-Nachweis)</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr">
+      <c r="G49" t="inlineStr">
         <is>
           <t>projektierer</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
         <is>
           <t>M+1</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr">
+      <c r="K49" t="inlineStr">
         <is>
           <t>keine</t>
         </is>

</xml_diff>

<commit_message>
Projektierung V4 Phase 93: Heizreport-API, UGL formatgenau, Stuecklisten-Pflege, v17
- heizreport_api: generischer REST-Client (Basis-URL, Auth header/bearer/basic/body,
  Endpunkte, Mapping hin/zurueck), Verbindungstest in den Einstellungen, Buttons
  Projekt anlegen / Ergebnis abrufen an der Heizlast-Aufgabe; Gewerk-Spalten
  heizreport_projekt_key, heizlast_quelle; docs/heizreport-api.md mit Anfragetext
- ugl.py nach UGL 4.0 (KOP/ADR/POA/POT/END, 200 Byte, cp850), Bestell-Dialog mit
  Vorschau, Lieferdatum, Lieferadresse, Bemerkung, Nachbestellung -2, Haekchen
  bei Collin hochgeladen; Tabelle ugl_bestellungen
- Parametrierung Stuecklisten: Pflege je Position mit Rueckschreiben ins Blatt
  (Backup), CSV Export/Import, Fortschritt, Go-live-Pruefpunkte; Spalte
  mengeneinheit; docs/ugl-format.md + docs/ugl-beispiel.ugl
- CLAUDE.md v17, docs/projektierung.md, Entscheidungen Phase 93; Tests Phase 93

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projektierung_logik_v1.xlsx
+++ b/projektierung_logik_v1.xlsx
@@ -5590,8 +5590,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -5619,6 +5622,11 @@
           <t>lieferant</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>mengeneinheit</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -5644,6 +5652,11 @@
           <t>Collin</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5669,6 +5682,11 @@
           <t>Collin</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5694,6 +5712,11 @@
           <t>Collin</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5719,6 +5742,11 @@
           <t>Collin</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5742,6 +5770,11 @@
       <c r="E6" t="inlineStr">
         <is>
           <t>Collin</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>ST</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
PLAN_PROJ_V3 Phase 84: Auftragsdaten fuer TAIFUN-Auftraege
- Zweite Seite Auftragsdaten nach Angebot -> Projekt (TAIFUN), Felder aus
  Blatt Steckbrief (neue Spalten eingabe/bezeichnung, quelle_typ auftragsdaten)
- Steckbrief-Werte mit quelle = auftragsdaten (nur FP-Erfassung ueberschreibt)
- Pflicht-PDF-Upload inkl. Galerie Allgemein und Projektablage
- Angebotsfeld kfw_gefoerdert (ja/nein/unbekannt), bza.ist_gefoerdert wertet es aus
- Button Auftragsdaten bearbeiten, Materialhinweis statt UGL bei TAIFUN
- steckbrief-abhaengige Paketschritte werden nachgezogen
- Stub auftragsdaten_aus_pdf; Abgleich-Vorspann im Plan
- Tests tests/test_projektierung_v3.py

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projektierung_logik_v1.xlsx
+++ b/projektierung_logik_v1.xlsx
@@ -4237,8 +4237,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:G87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -4266,6 +4270,16 @@
           <t>wert_oder_regel</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>eingabe</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>bezeichnung</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -5576,6 +5590,951 @@
       <c r="E52" t="inlineStr">
         <is>
           <t>*→{wert} m (laut Erfassung)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>hersteller</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>auswahl:Bosch|Mitsubishi|Vaillant|Sonstige</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Hersteller</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>serie_modell</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Serie/Modell</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>leistungsklasse</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>zahl</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Leistungsklasse (kW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>innengeraet</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Innengerät-Variante</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>puffer_l</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>zahl</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Puffer (l)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>warmwasser</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Warmwasser (Speicher l / über WP nein)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>aufstellort</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>auswahl:Boden|Wand|Garagendach|Fundament nötig</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Aufstellort Außengerät</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>zaehlerschrank</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>auswahl:bleibt|2-Feld|3-Feld|4-Feld</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Zählerschrank</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>unterverteilung</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Unterverteilung</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>alte_anlage</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>auswahl:Öl|Gas|Sonstige</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Alte Anlage</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>alte_anlage_standort</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Standort alte Anlage</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>oeltank</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Öltankentsorgung</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>oeltank_groesse</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>zahl</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Öltank: Größe (l)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>oeltank_material</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Öltank: Material/Zugang</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>stemmarbeiten</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Stemmarbeiten</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>erdleitung_m</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>zahl</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Erdleitung / Erdarbeiten (m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>dyn_tarif</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Dynamischer Tarif</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>imsys</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>iMSys</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>hems</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>HEMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>folierung</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Folierung</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>kran</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Materiallift/Kran</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>besonderheiten</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Besonderheiten</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>module_kwp</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Module (Anzahl, kWp)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>speicher</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>zahl</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Speicher (kWh)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>wechselrichter</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Wechselrichter</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>dach</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Dachtyp</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>geruest</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Gerüst nötig</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>wallbox</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>ja_nein</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Wallbox mit dabei</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>besonderheiten</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Besonderheiten</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>geraete</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>KL</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Gerät</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>anzahl</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>KL</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>zahl</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Anzahl</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>besonderheiten</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>KL</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Besonderheiten</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>geraet</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Wallbox (Gerät)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>anzahl</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>zahl</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Anzahl</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>besonderheiten</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>auftragsdaten</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Besonderheiten</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v28/v29-Nachtrag 08.10.2026: Antworten Andreas auf die Rückfragen des Durchlaufs
Nachtrag 2: WP ohne Sparten-Kopie (Standard-Vorlage gilt, Migration entfernt die
unveränderte Kopie), Streudatei anlagen/unternehmenspraesentation.pdf entfernt.

Projektierung (v28): volle Breite für alle main.breit-Seiten, Board-Mindesthöhe
auf kleinen Bildschirmen (kein Seiten-Scroll bei 1366x768), "Montage beenden" ohne
Kurzbericht, ib_kaeltemittel entfällt (30 Felder), migration_v28_entwuerfe leert
alte Formular-Entwürfe; bestätigte Annahmen dokumentiert.

Lead-Management (v29): HV-Direktlinks immer umleiten, "Mir zugeteilte Vorgänge"
vom Dashboard entfernt, Sperrzeiten exakt und durch Innendienst anlegbar,
Kundenantwort holt den Lead in die Kontaktierung, Admin-Glocke bei Mail-Status
fehler, Reply-To (Leadmanager + termin@), HV-Versandweg "entwurf" (.eml aus der
Vorschau, aus dem eigenen Postfach senden) als Standard.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projektierung_logik_v1.xlsx
+++ b/projektierung_logik_v1.xlsx
@@ -523,7 +523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G60"/>
+  <dimension ref="A1:G59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1342,27 +1342,27 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Gerät</t>
+          <t>Prüfungen</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ib_kaeltemittel</t>
+          <t>ib_f01</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Kältemittel / Füllmenge</t>
+          <t>1. Entsprechen Aufstellung und Montage den Herstellervorgaben, einschließlich Abständen, Schutzbereichen und gegebenenfalls Kondensatablauf?</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>ja_nein</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>J</t>
         </is>
       </c>
     </row>
@@ -1379,12 +1379,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ib_f01</t>
+          <t>ib_f02</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>1. Entsprechen Aufstellung und Montage den Herstellervorgaben, einschließlich Abständen, Schutzbereichen und gegebenenfalls Kondensatablauf?</t>
+          <t>2. Ist die Heizungsanlage gespült, befüllt, entlüftet und auf Dichtheit geprüft?</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1411,12 +1411,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ib_f02</t>
+          <t>ib_f03</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2. Ist die Heizungsanlage gespült, befüllt, entlüftet und auf Dichtheit geprüft?</t>
+          <t>3. Ist die Anlage mit Heizwasserqualität nach VDI2035 befüllt worden?</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1443,12 +1443,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ib_f03</t>
+          <t>ib_f04</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>3. Ist die Anlage mit Heizwasserqualität nach VDI2035 befüllt worden?</t>
+          <t>4. Ist der hydraulische Abgleich durchgeführt?</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1475,12 +1475,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ib_f04</t>
+          <t>ib_f05</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>4. Ist der hydraulische Abgleich durchgeführt?</t>
+          <t>5. Sind die herstellerseitig vorgesehenen Prüfungen an Sicherheitseinrichtungen, Frostschutz, Wärmequelle und Kältemittelkreis abgeschlossen?</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1507,12 +1507,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ib_f05</t>
+          <t>ib_f06</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>5. Sind die herstellerseitig vorgesehenen Prüfungen an Sicherheitseinrichtungen, Frostschutz, Wärmequelle und Kältemittelkreis abgeschlossen?</t>
+          <t>6. Sind Mindestvolumenstrom und erforderliches Anlagenwasservolumen sichergestellt?</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1539,22 +1539,27 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ib_f06</t>
+          <t>ib_f07_heizen</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>6. Sind Mindestvolumenstrom und erforderliches Anlagenwasservolumen sichergestellt?</t>
+          <t>7. Wurden die vorgesehenen Betriebsarten erfolgreich getestet? – Heizen</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ja_nein</t>
+          <t>auswahl</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
           <t>J</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>OK|nicht OK|nicht vorhanden</t>
         </is>
       </c>
     </row>
@@ -1571,12 +1576,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ib_f07_heizen</t>
+          <t>ib_f07_warmwasser</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>7. Wurden die vorgesehenen Betriebsarten erfolgreich getestet? – Heizen</t>
+          <t>7. Betriebsart Warmwasser</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1608,12 +1613,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ib_f07_warmwasser</t>
+          <t>ib_f07_kuehlen</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>7. Betriebsart Warmwasser</t>
+          <t>7. Betriebsart Kühlen</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1645,12 +1650,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ib_f07_kuehlen</t>
+          <t>ib_f07_zusatzheizung</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>7. Betriebsart Kühlen</t>
+          <t>7. Betriebsart Zusatzheizung</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1682,27 +1687,22 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ib_f07_zusatzheizung</t>
+          <t>ib_f08</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>7. Betriebsart Zusatzheizung</t>
+          <t>8. Sind die vereinbarten Steuerungs- und Kommunikationsschnittstellen eingerichtet und geprüft?</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>auswahl</t>
+          <t>ja_nein</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
           <t>J</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>OK|nicht OK|nicht vorhanden</t>
         </is>
       </c>
     </row>
@@ -1719,12 +1719,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ib_f08</t>
+          <t>ib_f09</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>8. Sind die vereinbarten Steuerungs- und Kommunikationsschnittstellen eingerichtet und geprüft?</t>
+          <t>9. Wurde der Betreiber in Bedienung, Störungsverhalten und Wartung eingewiesen und wurden die Unterlagen übergeben?</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1751,22 +1751,27 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ib_f09</t>
+          <t>ib_f10</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>9. Wurde der Betreiber in Bedienung, Störungsverhalten und Wartung eingewiesen und wurden die Unterlagen übergeben?</t>
+          <t>10. Welche Mängel oder Restarbeiten bestehen, wer erledigt sie und bis wann? (eine je Zeile, „keine“ erlaubt – wird als Restarbeiten-Liste übernommen)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ja_nein</t>
+          <t>text</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
           <t>J</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>gross</t>
         </is>
       </c>
     </row>
@@ -1783,17 +1788,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ib_f10</t>
+          <t>ib_f11</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>10. Welche Mängel oder Restarbeiten bestehen, wer erledigt sie und bis wann? (eine je Zeile, „keine“ erlaubt – wird als Restarbeiten-Liste übernommen)</t>
+          <t>11. Wird die Anlage durch den Techniker zum Betrieb freigegeben?</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>auswahl</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -1803,7 +1808,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>gross</t>
+          <t>Ja|Mit dokumentierten Einschränkungen|Nein</t>
         </is>
       </c>
     </row>
@@ -1820,27 +1825,27 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ib_f11</t>
+          <t>ib_f11_text</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>11. Wird die Anlage durch den Techniker zum Betrieb freigegeben?</t>
+          <t>Einschränkungen / Begründung</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>auswahl</t>
+          <t>text</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>N</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Ja|Mit dokumentierten Einschränkungen|Nein</t>
+          <t>pflicht_wenn:ib_f11≠Ja</t>
         </is>
       </c>
     </row>
@@ -1852,22 +1857,22 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Prüfungen</t>
+          <t>Betriebswerte im stabilen Betrieb</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ib_f11_text</t>
+          <t>ib_bw_betriebsart</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Einschränkungen / Begründung</t>
+          <t>Betriebsart</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>auswahl</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -1877,7 +1882,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>pflicht_wenn:ib_f11≠Ja</t>
+          <t>Heizen|Warmwasser|Kühlen</t>
         </is>
       </c>
     </row>
@@ -1894,27 +1899,22 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ib_bw_betriebsart</t>
+          <t>ib_bw_aussen</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Betriebsart</t>
+          <t>Außen-/Quellentemperatur (°C)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>auswahl</t>
+          <t>zahl</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
           <t>N</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Heizen|Warmwasser|Kühlen</t>
         </is>
       </c>
     </row>
@@ -1931,12 +1931,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ib_bw_aussen</t>
+          <t>ib_bw_druck</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Außen-/Quellentemperatur (°C)</t>
+          <t>Anlagendruck (bar)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1963,12 +1963,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ib_bw_druck</t>
+          <t>ib_bw_vorlauf</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Anlagendruck (bar)</t>
+          <t>Vorlauf (°C)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1995,12 +1995,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>ib_bw_vorlauf</t>
+          <t>ib_bw_ruecklauf</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Vorlauf (°C)</t>
+          <t>Rücklauf (°C)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2027,12 +2027,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ib_bw_ruecklauf</t>
+          <t>ib_bw_volumenstrom</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Rücklauf (°C)</t>
+          <t>Volumenstrom (l/min)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2054,22 +2054,22 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Betriebswerte im stabilen Betrieb</t>
+          <t>Einstellungen</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ib_bw_volumenstrom</t>
+          <t>ib_e_heizkurve</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Volumenstrom (l/min)</t>
+          <t>Heizkurve / Niveau</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>zahl</t>
+          <t>text</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2091,17 +2091,17 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>ib_e_heizkurve</t>
+          <t>ib_e_raumsoll</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Heizkurve / Niveau</t>
+          <t>Raum-Solltemperatur (°C)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>zahl</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2123,12 +2123,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ib_e_raumsoll</t>
+          <t>ib_e_wwsoll</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Raum-Solltemperatur (°C)</t>
+          <t>Warmwasser-Solltemperatur (°C)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2150,27 +2150,27 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Einstellungen</t>
+          <t>Unterschriften</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ib_e_wwsoll</t>
+          <t>ib_unterschrift_techniker</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Warmwasser-Solltemperatur (°C)</t>
+          <t>Unterschrift Techniker</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>zahl</t>
+          <t>unterschrift</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>J</t>
         </is>
       </c>
     </row>
@@ -2187,12 +2187,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ib_unterschrift_techniker</t>
+          <t>ib_unterschrift_betreiber</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Unterschrift Techniker</t>
+          <t>Betreiber – Einweisung und Unterlagenerhalt bestätigt</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2209,27 +2209,27 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>inbetriebnahme</t>
+          <t>abnahme</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Unterschriften</t>
+          <t>Leistung</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ib_unterschrift_betreiber</t>
+          <t>ab_vollstaendig</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Betreiber – Einweisung und Unterlagenerhalt bestätigt</t>
+          <t>Leistungen vollständig erbracht</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>unterschrift</t>
+          <t>ja_nein</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2251,22 +2251,22 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ab_vollstaendig</t>
+          <t>ab_maengel</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Leistungen vollständig erbracht</t>
+          <t>Mängel / Restarbeiten (eine je Zeile – wird als Restarbeiten-Liste übernommen)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>ja_nein</t>
+          <t>text</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -2283,22 +2283,27 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ab_maengel</t>
+          <t>ab_maengel_foto</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Mängel / Restarbeiten (eine je Zeile – wird als Restarbeiten-Liste übernommen)</t>
+          <t>Foto zu Mängeln</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>foto</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
           <t>N</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Inbetrieb-/Abnahme</t>
         </is>
       </c>
     </row>
@@ -2315,27 +2320,22 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ab_maengel_foto</t>
+          <t>ab_frist</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Foto zu Mängeln</t>
+          <t>Frist für Restarbeiten</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>foto</t>
+          <t>datum</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
           <t>N</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>Inbetrieb-/Abnahme</t>
         </is>
       </c>
     </row>
@@ -2347,27 +2347,27 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Leistung</t>
+          <t>Übergabe</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ab_frist</t>
+          <t>ab_unterlagen</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Frist für Restarbeiten</t>
+          <t>Unterlagen übergeben (Bedienungsanleitung, Garantie, Protokolle)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>datum</t>
+          <t>ja_nein</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>J</t>
         </is>
       </c>
     </row>
@@ -2384,12 +2384,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>ab_unterlagen</t>
+          <t>ab_einweisung_bestaetigt</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Unterlagen übergeben (Bedienungsanleitung, Garantie, Protokolle)</t>
+          <t>Kunde bestätigt Einweisung</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2411,22 +2411,22 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Übergabe</t>
+          <t>Unterschriften</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ab_einweisung_bestaetigt</t>
+          <t>ab_datum</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Kunde bestätigt Einweisung</t>
+          <t>Datum</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>ja_nein</t>
+          <t>datum</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2448,17 +2448,17 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ab_datum</t>
+          <t>ab_unterschrift_kunde</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Datum</t>
+          <t>Unterschrift Kunde</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>datum</t>
+          <t>unterschrift</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2480,12 +2480,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>ab_unterschrift_kunde</t>
+          <t>ab_unterschrift_monteur</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Unterschrift Kunde</t>
+          <t>Unterschrift Monteur</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2494,38 +2494,6 @@
         </is>
       </c>
       <c r="F59" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>abnahme</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Unterschriften</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>ab_unterschrift_monteur</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>Unterschrift Monteur</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>unterschrift</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
         <is>
           <t>J</t>
         </is>

</xml_diff>